<commit_message>
Adding pending clean files
</commit_message>
<xml_diff>
--- a/results/experiments_summary.xlsx
+++ b/results/experiments_summary.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\UMD Academic\NLP\nlp3\results\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83FDF8FA-C447-45C5-BE09-D21C3F534240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="31">
   <si>
     <t>Model</t>
   </si>
@@ -65,9 +71,6 @@
   </si>
   <si>
     <t>0.4993</t>
-  </si>
-  <si>
-    <t>0.3330</t>
   </si>
   <si>
     <t>129.83</t>
@@ -115,8 +118,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,13 +182,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -223,7 +234,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -257,6 +268,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -291,9 +303,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -466,11 +479,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -502,7 +515,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -519,22 +532,22 @@
         <v>14</v>
       </c>
       <c r="F2">
-        <v>0.7297</v>
+        <v>0.72970000000000002</v>
       </c>
       <c r="G2">
-        <v>0.7297</v>
+        <v>0.72970000000000002</v>
       </c>
       <c r="H2">
         <v>60.15</v>
       </c>
       <c r="I2">
-        <v>0.3708</v>
+        <v>0.37080000000000002</v>
       </c>
       <c r="J2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -551,22 +564,22 @@
         <v>15</v>
       </c>
       <c r="F3">
-        <v>0.7256</v>
+        <v>0.72560000000000002</v>
       </c>
       <c r="G3">
-        <v>0.7251</v>
+        <v>0.72509999999999997</v>
       </c>
       <c r="H3">
         <v>50.81</v>
       </c>
       <c r="I3">
-        <v>0.3672</v>
+        <v>0.36720000000000003</v>
       </c>
       <c r="J3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -583,22 +596,22 @@
         <v>14</v>
       </c>
       <c r="F4">
-        <v>0.7808</v>
+        <v>0.78080000000000005</v>
       </c>
       <c r="G4">
-        <v>0.7808</v>
+        <v>0.78080000000000005</v>
       </c>
       <c r="H4">
         <v>85.5</v>
       </c>
       <c r="I4">
-        <v>0.3184</v>
+        <v>0.31840000000000002</v>
       </c>
       <c r="J4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -615,22 +628,22 @@
         <v>15</v>
       </c>
       <c r="F5">
-        <v>0.7803</v>
+        <v>0.78029999999999999</v>
       </c>
       <c r="G5">
-        <v>0.7803</v>
+        <v>0.78029999999999999</v>
       </c>
       <c r="H5">
         <v>78.19</v>
       </c>
       <c r="I5">
-        <v>0.3107</v>
+        <v>0.31069999999999998</v>
       </c>
       <c r="J5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -647,22 +660,22 @@
         <v>14</v>
       </c>
       <c r="F6">
-        <v>0.8339</v>
+        <v>0.83389999999999997</v>
       </c>
       <c r="G6">
-        <v>0.8339</v>
+        <v>0.83389999999999997</v>
       </c>
       <c r="H6">
-        <v>147.39</v>
+        <v>147.38999999999999</v>
       </c>
       <c r="I6">
-        <v>0.2628</v>
+        <v>0.26279999999999998</v>
       </c>
       <c r="J6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -679,22 +692,22 @@
         <v>15</v>
       </c>
       <c r="F7">
-        <v>0.8328</v>
+        <v>0.83279999999999998</v>
       </c>
       <c r="G7">
         <v>0.8327</v>
       </c>
       <c r="H7">
-        <v>150.33</v>
+        <v>150.33000000000001</v>
       </c>
       <c r="I7">
-        <v>0.262</v>
+        <v>0.26200000000000001</v>
       </c>
       <c r="J7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -711,22 +724,22 @@
         <v>14</v>
       </c>
       <c r="F8">
-        <v>0.5116000000000001</v>
+        <v>0.51160000000000005</v>
       </c>
       <c r="G8">
-        <v>0.5014</v>
+        <v>0.50139999999999996</v>
       </c>
       <c r="H8">
         <v>45.14</v>
       </c>
       <c r="I8">
-        <v>0.6935</v>
+        <v>0.69350000000000001</v>
       </c>
       <c r="J8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -743,22 +756,22 @@
         <v>15</v>
       </c>
       <c r="F9">
-        <v>0.5033</v>
+        <v>0.50329999999999997</v>
       </c>
       <c r="G9">
-        <v>0.3608</v>
+        <v>0.49080000000000001</v>
       </c>
       <c r="H9">
         <v>45.36</v>
       </c>
       <c r="I9">
-        <v>0.6936</v>
+        <v>0.69359999999999999</v>
       </c>
       <c r="J9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -775,22 +788,22 @@
         <v>14</v>
       </c>
       <c r="F10">
-        <v>0.5006</v>
+        <v>0.50060000000000004</v>
       </c>
       <c r="G10">
-        <v>0.3337</v>
+        <v>0.59370000000000001</v>
       </c>
       <c r="H10">
         <v>82.39</v>
       </c>
       <c r="I10">
-        <v>0.6935</v>
+        <v>0.69350000000000001</v>
       </c>
       <c r="J10" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -807,22 +820,22 @@
         <v>15</v>
       </c>
       <c r="F11">
-        <v>0.4998</v>
+        <v>0.49980000000000002</v>
       </c>
       <c r="G11">
-        <v>0.3382</v>
+        <v>0.59819999999999995</v>
       </c>
       <c r="H11">
         <v>81.83</v>
       </c>
       <c r="I11">
-        <v>0.6932</v>
+        <v>0.69320000000000004</v>
       </c>
       <c r="J11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -839,22 +852,22 @@
         <v>14</v>
       </c>
       <c r="F12">
-        <v>0.4993</v>
+        <v>0.49930000000000002</v>
       </c>
       <c r="G12">
-        <v>0.333</v>
+        <v>0.63300000000000001</v>
       </c>
       <c r="H12">
         <v>133.5</v>
       </c>
       <c r="I12">
-        <v>0.6934</v>
+        <v>0.69340000000000002</v>
       </c>
       <c r="J12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -873,17 +886,17 @@
       <c r="F13" t="s">
         <v>16</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13">
+        <v>0.63300000000000001</v>
+      </c>
+      <c r="H13" t="s">
         <v>17</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>18</v>
       </c>
-      <c r="I13" t="s">
-        <v>19</v>
-      </c>
       <c r="J13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>